<commit_message>
chore: update northbound mutual fund AUM
</commit_message>
<xml_diff>
--- a/outputs/latest.xlsx
+++ b/outputs/latest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合并成基金全称" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分各个份额（仅内地销售份额，不含所有份额）" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="合并成基金全称" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="分各个份额（仅内地销售份额，不含所有份额）" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'合并成基金全称'!$A$1:$T$45</definedName>
@@ -163,203 +163,203 @@
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J3" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 建银国际资管
-抓取信息: Link discovery failed for https://www.ccbintl.com.hk/English/management7.html: HTTPSConnectionPool(host='www.ccbintl.com.hk', port=443): Max retries exceeded with url: /English/management7.html (Caused by SSLError(SSLCertVerificationError(1, '[SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: unable to get local issuer certificate (_ssl.c:1010)'))) | Fetch failed for https://www.ccbintl.com.hk/English/management7.html: HTTPSConnectionPool(host='www.ccbintl.com.hk', port=443): Max retries exceeded with url: /English/management7.html (Caused by SSLError(SSLCertVerificationError(1, '[SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: unable to get local issuer certificate (_ssl</t>
+抓取信息: No manager source configured for 建银国际资管.</t>
       </text>
     </comment>
     <comment ref="J4" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 中银香港资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 中银香港资管.</t>
       </text>
     </comment>
     <comment ref="J5" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 中银香港资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 中银香港资管.</t>
       </text>
     </comment>
     <comment ref="J6" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 行健资管
-抓取信息: Link discovery failed for https://www.zealasset.com/en/about-us: HTTPSConnectionPool(host='www.zealasset.com', port=443): Max retries exceeded with url: /en/about-us (Caused by SSLError(SSLEOFError(8, '[SSL: UNEXPECTED_EOF_WHILE_READING] EOF occurred in violation of protocol (_ssl.c:1010)'))) | Fetch failed for https://www.zealasset.com/en/about-us: HTTPSConnectionPool(host='www.zealasset.com', port=443): Max retries exceeded with url: /en/about-us (Caused by SSLError(SSLEOFError(8, '[SSL: UNEXPECTED_EOF_WHILE_READING] EOF occurred in violation of protocol (_ssl.c:1010)'))) | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 行健资管.</t>
       </text>
     </comment>
     <comment ref="J7" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 中银保诚资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 中银保诚资管.</t>
       </text>
     </comment>
     <comment ref="J8" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 中银保诚资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 中银保诚资管.</t>
       </text>
     </comment>
     <comment ref="J9" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 恒生投资管理
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 恒生投资管理.</t>
       </text>
     </comment>
     <comment ref="J10" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J11" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J12" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 中银香港资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 中银香港资管.</t>
       </text>
     </comment>
     <comment ref="J13" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 施罗德投资管理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 施罗德投资管理(香港).</t>
       </text>
     </comment>
     <comment ref="J14" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J15" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 恒生投资管理
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 恒生投资管理.</t>
       </text>
     </comment>
     <comment ref="J16" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J17" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J18" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J19" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J20" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J21" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J22" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 海通国际资管(香港)
-抓取信息: Link discovery failed for https://www.haitongetf.com.hk/asm/en-us: HTTPSConnectionPool(host='www.haitongetf.com.hk', port=443): Max retries exceeded with url: /asm/en-us (Caused by SSLError(SSLCertVerificationError(1, "[SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: Hostname mismatch, certificate is not valid for 'www.haitongetf.com.hk'. (_ssl.c:1010)"))) | Fetch failed for https://www.haitongetf.com.hk/asm/en-us: HTTPSConnectionPool(host='www.haitongetf.com.hk', port=443): Max retries exceeded with url: /asm/en-us (Caused by SSLError(SSLCertVerificationError(1, "[SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: Hostname mismatch, certificate is not valid for 'www.haito</t>
+抓取信息: No manager source configured for 海通国际资管(香港).</t>
       </text>
     </comment>
     <comment ref="J23" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J24" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 博时基金(国际)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 博时基金(国际).</t>
       </text>
     </comment>
     <comment ref="J25" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J26" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J27" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J28" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J29" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J30" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J31" authorId="0" shapeId="0">
@@ -371,98 +371,98 @@
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 易方达资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 易方达资管(香港).</t>
       </text>
     </comment>
     <comment ref="J33" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J34" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 弘收资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 弘收资管(香港).</t>
       </text>
     </comment>
     <comment ref="J35" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 高腾国际资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 高腾国际资管.</t>
       </text>
     </comment>
     <comment ref="J36" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 兴证国际资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 兴证国际资管.</t>
       </text>
     </comment>
     <comment ref="J37" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银基金(卢森堡)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银基金(卢森堡).</t>
       </text>
     </comment>
     <comment ref="J38" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J39" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 南方东英资管
-抓取信息: Link discovery failed for https://www.csopasset.com/: 403 Client Error: Forbidden for url: https://www.csopasset.com/ | Fetch failed for https://www.csopasset.com/: 403 Client Error: Forbidden for url: https://www.csopasset.com/ | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 南方东英资管.</t>
       </text>
     </comment>
     <comment ref="J40" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J41" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根资管(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根资管(亚太).</t>
       </text>
     </comment>
     <comment ref="J42" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J43" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J44" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J45" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
   </commentList>
@@ -479,441 +479,441 @@
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J3" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J4" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J5" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J6" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 行健资管
-抓取信息: Link discovery failed for https://www.zealasset.com/en/about-us: HTTPSConnectionPool(host='www.zealasset.com', port=443): Max retries exceeded with url: /en/about-us (Caused by SSLError(SSLEOFError(8, '[SSL: UNEXPECTED_EOF_WHILE_READING] EOF occurred in violation of protocol (_ssl.c:1010)'))) | Fetch failed for https://www.zealasset.com/en/about-us: HTTPSConnectionPool(host='www.zealasset.com', port=443): Max retries exceeded with url: /en/about-us (Caused by SSLError(SSLEOFError(8, '[SSL: UNEXPECTED_EOF_WHILE_READING] EOF occurred in violation of protocol (_ssl.c:1010)'))) | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 行健资管.</t>
       </text>
     </comment>
     <comment ref="J7" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 恒生投资管理
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 恒生投资管理.</t>
       </text>
     </comment>
     <comment ref="J8" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 恒生投资管理
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 恒生投资管理.</t>
       </text>
     </comment>
     <comment ref="J9" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 建银国际资管
-抓取信息: Link discovery failed for https://www.ccbintl.com.hk/English/management7.html: HTTPSConnectionPool(host='www.ccbintl.com.hk', port=443): Max retries exceeded with url: /English/management7.html (Caused by SSLError(SSLCertVerificationError(1, '[SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: unable to get local issuer certificate (_ssl.c:1010)'))) | Fetch failed for https://www.ccbintl.com.hk/English/management7.html: HTTPSConnectionPool(host='www.ccbintl.com.hk', port=443): Max retries exceeded with url: /English/management7.html (Caused by SSLError(SSLCertVerificationError(1, '[SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: unable to get local issuer certificate (_ssl</t>
+抓取信息: No manager source configured for 建银国际资管.</t>
       </text>
     </comment>
     <comment ref="J10" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J11" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J12" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 中银香港资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 中银香港资管.</t>
       </text>
     </comment>
     <comment ref="J13" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 施罗德投资管理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 施罗德投资管理(香港).</t>
       </text>
     </comment>
     <comment ref="J14" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J15" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J16" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J17" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J18" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J19" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J20" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 中银保诚资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 中银保诚资管.</t>
       </text>
     </comment>
     <comment ref="J21" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J22" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 恒生投资管理
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 恒生投资管理.</t>
       </text>
     </comment>
     <comment ref="J23" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 中银保诚资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 中银保诚资管.</t>
       </text>
     </comment>
     <comment ref="J24" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 中银香港资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 中银香港资管.</t>
       </text>
     </comment>
     <comment ref="J25" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J26" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J27" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J28" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J29" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J30" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J31" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J32" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J33" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J34" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J35" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J36" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J37" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J38" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J39" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J40" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J41" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J42" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J43" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J44" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J45" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J46" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J47" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J48" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J49" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 海通国际资管(香港)
-抓取信息: Link discovery failed for https://www.haitongetf.com.hk/asm/en-us: HTTPSConnectionPool(host='www.haitongetf.com.hk', port=443): Max retries exceeded with url: /asm/en-us (Caused by SSLError(SSLCertVerificationError(1, "[SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: Hostname mismatch, certificate is not valid for 'www.haitongetf.com.hk'. (_ssl.c:1010)"))) | Fetch failed for https://www.haitongetf.com.hk/asm/en-us: HTTPSConnectionPool(host='www.haitongetf.com.hk', port=443): Max retries exceeded with url: /asm/en-us (Caused by SSLError(SSLCertVerificationError(1, "[SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: Hostname mismatch, certificate is not valid for 'www.haito</t>
+抓取信息: No manager source configured for 海通国际资管(香港).</t>
       </text>
     </comment>
     <comment ref="J50" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 博时基金(国际)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 博时基金(国际).</t>
       </text>
     </comment>
     <comment ref="J51" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 博时基金(国际)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 博时基金(国际).</t>
       </text>
     </comment>
     <comment ref="J52" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 博时基金(国际)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 博时基金(国际).</t>
       </text>
     </comment>
     <comment ref="J53" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 博时基金(国际)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 博时基金(国际).</t>
       </text>
     </comment>
     <comment ref="J54" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J55" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J56" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J57" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J58" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J59" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J60" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J61" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J62" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J63" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J64" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J65" authorId="0" shapeId="0">
@@ -930,469 +930,469 @@
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J68" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J69" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J70" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J71" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J72" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J73" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J74" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J75" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J76" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J77" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J78" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J79" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J80" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J81" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J82" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J83" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J84" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J85" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J86" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J87" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J88" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J89" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J90" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J91" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J92" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J93" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J94" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J95" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J96" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 海通国际资管(香港)
-抓取信息: Link discovery failed for https://www.haitongetf.com.hk/asm/en-us: HTTPSConnectionPool(host='www.haitongetf.com.hk', port=443): Max retries exceeded with url: /asm/en-us (Caused by SSLError(SSLCertVerificationError(1, "[SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: Hostname mismatch, certificate is not valid for 'www.haitongetf.com.hk'. (_ssl.c:1010)"))) | Fetch failed for https://www.haitongetf.com.hk/asm/en-us: HTTPSConnectionPool(host='www.haitongetf.com.hk', port=443): Max retries exceeded with url: /asm/en-us (Caused by SSLError(SSLCertVerificationError(1, "[SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: Hostname mismatch, certificate is not valid for 'www.haito</t>
+抓取信息: No manager source configured for 海通国际资管(香港).</t>
       </text>
     </comment>
     <comment ref="J97" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 海通国际资管(香港)
-抓取信息: Link discovery failed for https://www.haitongetf.com.hk/asm/en-us: HTTPSConnectionPool(host='www.haitongetf.com.hk', port=443): Max retries exceeded with url: /asm/en-us (Caused by SSLError(SSLCertVerificationError(1, "[SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: Hostname mismatch, certificate is not valid for 'www.haitongetf.com.hk'. (_ssl.c:1010)"))) | Fetch failed for https://www.haitongetf.com.hk/asm/en-us: HTTPSConnectionPool(host='www.haitongetf.com.hk', port=443): Max retries exceeded with url: /asm/en-us (Caused by SSLError(SSLCertVerificationError(1, "[SSL: CERTIFICATE_VERIFY_FAILED] certificate verify failed: Hostname mismatch, certificate is not valid for 'www.haito</t>
+抓取信息: No manager source configured for 海通国际资管(香港).</t>
       </text>
     </comment>
     <comment ref="J98" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J99" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J100" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J101" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 易方达资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 易方达资管(香港).</t>
       </text>
     </comment>
     <comment ref="J102" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 易方达资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 易方达资管(香港).</t>
       </text>
     </comment>
     <comment ref="J103" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 易方达资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 易方达资管(香港).</t>
       </text>
     </comment>
     <comment ref="J104" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 弘收资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 弘收资管(香港).</t>
       </text>
     </comment>
     <comment ref="J105" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 弘收资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 弘收资管(香港).</t>
       </text>
     </comment>
     <comment ref="J106" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 弘收资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 弘收资管(香港).</t>
       </text>
     </comment>
     <comment ref="J107" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 弘收资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 弘收资管(香港).</t>
       </text>
     </comment>
     <comment ref="J108" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 高腾国际资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 高腾国际资管.</t>
       </text>
     </comment>
     <comment ref="J109" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 高腾国际资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 高腾国际资管.</t>
       </text>
     </comment>
     <comment ref="J110" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 高腾国际资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 高腾国际资管.</t>
       </text>
     </comment>
     <comment ref="J111" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 高腾国际资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 高腾国际资管.</t>
       </text>
     </comment>
     <comment ref="J112" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J113" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J114" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J115" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 兴证国际资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 兴证国际资管.</t>
       </text>
     </comment>
     <comment ref="J116" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 高腾国际资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 高腾国际资管.</t>
       </text>
     </comment>
     <comment ref="J117" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 高腾国际资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 高腾国际资管.</t>
       </text>
     </comment>
     <comment ref="J118" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银基金(卢森堡)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银基金(卢森堡).</t>
       </text>
     </comment>
     <comment ref="J119" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 中银香港资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 中银香港资管.</t>
       </text>
     </comment>
     <comment ref="J120" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 南方东英资管
-抓取信息: Link discovery failed for https://www.csopasset.com/: 403 Client Error: Forbidden for url: https://www.csopasset.com/ | Fetch failed for https://www.csopasset.com/: 403 Client Error: Forbidden for url: https://www.csopasset.com/ | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 南方东英资管.</t>
       </text>
     </comment>
     <comment ref="J121" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 中银香港资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 中银香港资管.</t>
       </text>
     </comment>
     <comment ref="J122" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 中银香港资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 中银香港资管.</t>
       </text>
     </comment>
     <comment ref="J123" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J124" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J125" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根资管(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根资管(亚太).</t>
       </text>
     </comment>
     <comment ref="J126" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根资管(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根资管(亚太).</t>
       </text>
     </comment>
     <comment ref="J127" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根资管(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根资管(亚太).</t>
       </text>
     </comment>
     <comment ref="J128" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J129" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J130" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J131" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 施罗德投资管理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 施罗德投资管理(香港).</t>
       </text>
     </comment>
     <comment ref="J132" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 施罗德投资管理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 施罗德投资管理(香港).</t>
       </text>
     </comment>
     <comment ref="J133" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 施罗德投资管理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 施罗德投资管理(香港).</t>
       </text>
     </comment>
     <comment ref="J134" authorId="0" shapeId="0">
@@ -1404,42 +1404,42 @@
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J136" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东亚联丰投资管理
-抓取信息: Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202601_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FABC_commentary_202604_EN_Final.pdf: Stream has ended unexpectedly | Fetch failed for https://www.buim.com/get_pdf.php?pdf=images%2Fdata%2FFund_Commentary%2F2026%2FAPM_commentary_202603_EN_Final.pdf: Stream has ended unexpectedly</t>
+抓取信息: No manager source configured for 东亚联丰投资管理.</t>
       </text>
     </comment>
     <comment ref="J137" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J138" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J139" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J140" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J141" authorId="0" shapeId="0">
@@ -1456,749 +1456,749 @@
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J144" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J145" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J146" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J147" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J148" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 汇丰投资基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 汇丰投资基金(香港).</t>
       </text>
     </comment>
     <comment ref="J149" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J150" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J151" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J152" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J153" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J154" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J155" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J156" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 东方汇理(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 东方汇理(香港).</t>
       </text>
     </comment>
     <comment ref="J157" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 中银保诚资管
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 中银保诚资管.</t>
       </text>
     </comment>
     <comment ref="J158" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J159" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J160" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J161" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J162" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J163" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J164" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J165" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J166" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 摩根基金(亚洲)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 摩根基金(亚洲).</t>
       </text>
     </comment>
     <comment ref="J167" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 安联环球投资(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 安联环球投资(亚太).</t>
       </text>
     </comment>
     <comment ref="J168" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 安联环球投资(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 安联环球投资(亚太).</t>
       </text>
     </comment>
     <comment ref="J169" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 安联环球投资(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 安联环球投资(亚太).</t>
       </text>
     </comment>
     <comment ref="J170" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 安联环球投资(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 安联环球投资(亚太).</t>
       </text>
     </comment>
     <comment ref="J171" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 安联环球投资(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 安联环球投资(亚太).</t>
       </text>
     </comment>
     <comment ref="J172" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 安联环球投资(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 安联环球投资(亚太).</t>
       </text>
     </comment>
     <comment ref="J173" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 安联环球投资(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 安联环球投资(亚太).</t>
       </text>
     </comment>
     <comment ref="J174" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 安联环球投资(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 安联环球投资(亚太).</t>
       </text>
     </comment>
     <comment ref="J175" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 安联环球投资(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 安联环球投资(亚太).</t>
       </text>
     </comment>
     <comment ref="J176" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 安联环球投资(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 安联环球投资(亚太).</t>
       </text>
     </comment>
     <comment ref="J177" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 安联环球投资(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 安联环球投资(亚太).</t>
       </text>
     </comment>
     <comment ref="J178" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 安联环球投资(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 安联环球投资(亚太).</t>
       </text>
     </comment>
     <comment ref="J179" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 安联环球投资(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 安联环球投资(亚太).</t>
       </text>
     </comment>
     <comment ref="J180" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 安联环球投资(亚太)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 安联环球投资(亚太).</t>
       </text>
     </comment>
     <comment ref="J181" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J182" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J183" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J184" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J185" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J186" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J187" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J188" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J189" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J190" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J191" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J192" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J193" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J194" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J195" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J196" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J197" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J198" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J199" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J200" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 华夏基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 华夏基金(香港).</t>
       </text>
     </comment>
     <comment ref="J201" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 贝莱德资管(北亚)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 贝莱德资管(北亚).</t>
       </text>
     </comment>
     <comment ref="J202" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 贝莱德资管(北亚)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 贝莱德资管(北亚).</t>
       </text>
     </comment>
     <comment ref="J203" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 贝莱德资管(北亚)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 贝莱德资管(北亚).</t>
       </text>
     </comment>
     <comment ref="J204" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 太平资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 太平资管(香港).</t>
       </text>
     </comment>
     <comment ref="J205" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 易方达资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 易方达资管(香港).</t>
       </text>
     </comment>
     <comment ref="J206" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 易方达资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 易方达资管(香港).</t>
       </text>
     </comment>
     <comment ref="J207" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 易方达资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 易方达资管(香港).</t>
       </text>
     </comment>
     <comment ref="J208" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 易方达资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 易方达资管(香港).</t>
       </text>
     </comment>
     <comment ref="J209" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 易方达资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 易方达资管(香港).</t>
       </text>
     </comment>
     <comment ref="J210" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 易方达资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 易方达资管(香港).</t>
       </text>
     </comment>
     <comment ref="J211" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 易方达资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 易方达资管(香港).</t>
       </text>
     </comment>
     <comment ref="J212" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 易方达资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 易方达资管(香港).</t>
       </text>
     </comment>
     <comment ref="J213" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 易方达资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 易方达资管(香港).</t>
       </text>
     </comment>
     <comment ref="J214" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 易方达资管(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 易方达资管(香港).</t>
       </text>
     </comment>
     <comment ref="J215" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 富达基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 富达基金(香港).</t>
       </text>
     </comment>
     <comment ref="J216" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 富达基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 富达基金(香港).</t>
       </text>
     </comment>
     <comment ref="J217" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 富达基金(香港)
-抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No manager source configured for 富达基金(香港).</t>
       </text>
     </comment>
     <comment ref="J218" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J219" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J220" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J221" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J222" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J223" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J224" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J225" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J226" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J227" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J228" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J229" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J230" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J231" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J232" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J233" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J234" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J235" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 瑞银环球资管(香港)
-抓取信息: Link discovery failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | Fetch failed for https://www.ubs.com/hk/en/assetmanagement: 403 Client Error: Forbidden for url: https://www.ubs.com/hk/en/assetmanagement | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 瑞银环球资管(香港).</t>
       </text>
     </comment>
     <comment ref="J236" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J237" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J238" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J239" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J240" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J241" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J242" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J243" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J244" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J245" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J246" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J247" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J248" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
     <comment ref="J249" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: No manager source configured for 惠理基金(香港).</t>
       </text>
     </comment>
   </commentList>

</xml_diff>